<commit_message>
Store Datum verzameld as real dates, fix L0001 opmerking wording
Datum verzameld is now written as an actual Excel date (not text) in
both the pilot import script and the regenerated pilot file, so future
sorting and filtering by date works correctly; the visible dd-mm-jjjj
notation is unchanged. Also replaces one sentence in the L0001
Opmerkingen field to describe the ~2.000 employee figure directly
instead of referencing a source margin. No other values, segments,
sources, dropdowns or columns changed; the original template is
untouched.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Pna7MwDh3vF9ehMRt2WXJn
</commit_message>
<xml_diff>
--- a/data/HAHEBO_leadbestand_pilot.xlsx
+++ b/data/HAHEBO_leadbestand_pilot.xlsx
@@ -712,14 +712,12 @@
           <t>nog niet gecontroleerd</t>
         </is>
       </c>
-      <c r="Y2" s="3" t="inlineStr">
-        <is>
-          <t>15-09-2026</t>
-        </is>
+      <c r="Y2" s="3" t="n">
+        <v>46280</v>
       </c>
       <c r="Z2" t="inlineStr">
         <is>
-          <t>Segment toegekend op basis van een actuele locatiepagina zonder expliciete peildatum. Het aantal valt met de eigen marge van de bron volledig in het bereik 50 of meer. Eerder gevonden afwijkende cijfers veranderen dit niet: circa 1.400 betreft heel Nederland en valt af op meetniveau, circa 2.100 komt uit een C-bron en wijst dezelfde kant op. Geen algemeen e-mailadres gepubliceerd, alleen een adres voor orderverwerking. Naast het NL-domein bestaat ook een .com-domein.</t>
+          <t>Segment toegekend op basis van een actuele locatiepagina zonder expliciete peildatum. De bron noemt ongeveer 2.000 medewerkers op de locatie; dit ligt eenduidig in het segment 50+. Eerder gevonden afwijkende cijfers veranderen dit niet: circa 1.400 betreft heel Nederland en valt af op meetniveau, circa 2.100 komt uit een C-bron en wijst dezelfde kant op. Geen algemeen e-mailadres gepubliceerd, alleen een adres voor orderverwerking. Naast het NL-domein bestaat ook een .com-domein.</t>
         </is>
       </c>
     </row>
@@ -834,10 +832,8 @@
           <t>nog niet gecontroleerd</t>
         </is>
       </c>
-      <c r="Y3" s="3" t="inlineStr">
-        <is>
-          <t>15-09-2026</t>
-        </is>
+      <c r="Y3" s="3" t="n">
+        <v>46280</v>
       </c>
       <c r="Z3" t="inlineStr">
         <is>
@@ -956,10 +952,8 @@
           <t>nog niet gecontroleerd</t>
         </is>
       </c>
-      <c r="Y4" s="3" t="inlineStr">
-        <is>
-          <t>15-09-2026</t>
-        </is>
+      <c r="Y4" s="3" t="n">
+        <v>46280</v>
       </c>
       <c r="Z4" t="inlineStr">
         <is>
@@ -1078,10 +1072,8 @@
           <t>nog niet gecontroleerd</t>
         </is>
       </c>
-      <c r="Y5" s="3" t="inlineStr">
-        <is>
-          <t>15-09-2026</t>
-        </is>
+      <c r="Y5" s="3" t="n">
+        <v>46280</v>
       </c>
       <c r="Z5" t="inlineStr">
         <is>
@@ -1200,10 +1192,8 @@
           <t>nog niet gecontroleerd</t>
         </is>
       </c>
-      <c r="Y6" s="3" t="inlineStr">
-        <is>
-          <t>15-09-2026</t>
-        </is>
+      <c r="Y6" s="3" t="n">
+        <v>46280</v>
       </c>
       <c r="Z6" t="inlineStr">
         <is>

</xml_diff>